<commit_message>
correct data on steel
</commit_message>
<xml_diff>
--- a/src/cassy/additional_data/materials/SS316L(N)-IG.xlsx
+++ b/src/cassy/additional_data/materials/SS316L(N)-IG.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Analyses\F4E-OMF-1091\Task#3\PbLi\KAISER-Developing\src\kaiser\additional_data\materials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\src\cassy\additional_data\materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02BEDE2-DBB2-415C-BF14-4BC8FCA59DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="715" activeTab="8"/>
+    <workbookView xWindow="4466" yWindow="3171" windowWidth="21600" windowHeight="11195" tabRatio="715" firstSheet="5" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sd_nopeak" sheetId="13" r:id="rId1"/>
@@ -30,7 +31,7 @@
     <sheet name="TrueStressStrain" sheetId="14" r:id="rId16"/>
     <sheet name="TrueStressStrain2" sheetId="15" r:id="rId17"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,6 +44,7 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -192,7 +194,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -1239,7 +1241,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1550,19 +1552,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A2" s="55"/>
       <c r="B2" s="81" t="s">
         <v>16</v>
@@ -1578,7 +1580,7 @@
       <c r="K2" s="81"/>
       <c r="L2" s="81"/>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="65" t="s">
         <v>13</v>
       </c>
@@ -1616,7 +1618,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="69">
         <v>20</v>
       </c>
@@ -1654,7 +1656,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A5" s="70">
         <v>50</v>
       </c>
@@ -1692,7 +1694,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A6" s="70">
         <v>100</v>
       </c>
@@ -1730,7 +1732,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="70">
         <v>150</v>
       </c>
@@ -1768,7 +1770,7 @@
         <v>411.02</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="70">
         <v>200</v>
       </c>
@@ -1806,7 +1808,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="70">
         <v>250</v>
       </c>
@@ -1844,7 +1846,7 @@
         <v>449.01</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="70">
         <v>300</v>
       </c>
@@ -1882,7 +1884,7 @@
         <v>449.02</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="71">
         <v>350</v>
       </c>
@@ -1929,19 +1931,19 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A2" s="55"/>
       <c r="B2" s="81" t="s">
         <v>16</v>
@@ -1957,7 +1959,7 @@
       <c r="K2" s="81"/>
       <c r="L2" s="81"/>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="65" t="s">
         <v>13</v>
       </c>
@@ -1995,7 +1997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="69">
         <v>20</v>
       </c>
@@ -2033,7 +2035,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A5" s="70">
         <v>50</v>
       </c>
@@ -2071,7 +2073,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A6" s="70">
         <v>100</v>
       </c>
@@ -2109,7 +2111,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="70">
         <v>150</v>
       </c>
@@ -2147,7 +2149,7 @@
         <v>411.02</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="70">
         <v>200</v>
       </c>
@@ -2185,7 +2187,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="70">
         <v>250</v>
       </c>
@@ -2223,7 +2225,7 @@
         <v>449.01</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="70">
         <v>300</v>
       </c>
@@ -2261,7 +2263,7 @@
         <v>449.02</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="71">
         <v>350</v>
       </c>
@@ -2308,16 +2310,16 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A2" s="55"/>
       <c r="B2" s="81" t="s">
         <v>15</v>
@@ -2333,7 +2335,7 @@
       <c r="K2" s="81"/>
       <c r="L2" s="81"/>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="65" t="s">
         <v>13</v>
       </c>
@@ -2371,7 +2373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="69">
         <v>20</v>
       </c>
@@ -2409,7 +2411,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A5" s="70">
         <v>50</v>
       </c>
@@ -2447,7 +2449,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A6" s="70">
         <v>100</v>
       </c>
@@ -2485,7 +2487,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="70">
         <v>150</v>
       </c>
@@ -2523,7 +2525,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="70">
         <v>200</v>
       </c>
@@ -2561,7 +2563,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="70">
         <v>250</v>
       </c>
@@ -2599,7 +2601,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="70">
         <v>300</v>
       </c>
@@ -2637,7 +2639,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="71">
         <v>350</v>
       </c>
@@ -2685,14 +2687,14 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:O4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="13" t="s">
         <v>9</v>
       </c>
@@ -2713,7 +2715,7 @@
       <c r="N1" s="91"/>
       <c r="O1" s="91"/>
     </row>
-    <row r="2" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
@@ -2760,7 +2762,7 @@
         <v>1400000000</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A3" s="18">
         <v>20</v>
       </c>
@@ -2807,7 +2809,7 @@
         <v>1.88</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="21">
         <v>450</v>
       </c>
@@ -2863,14 +2865,14 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:O4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -2891,7 +2893,7 @@
       <c r="N1" s="93"/>
       <c r="O1" s="93"/>
     </row>
-    <row r="2" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
@@ -2938,7 +2940,7 @@
         <v>1400000000</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A3" s="18">
         <v>20</v>
       </c>
@@ -2985,7 +2987,7 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="26">
         <v>450</v>
       </c>
@@ -3041,15 +3043,15 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="12.28515625" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="2" width="12.3046875" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -3060,7 +3062,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="32">
         <v>20</v>
       </c>
@@ -3071,7 +3073,7 @@
         <v>0.3387</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>450</v>
       </c>
@@ -3082,7 +3084,7 @@
         <v>0.30249999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="35">
         <v>600</v>
       </c>
@@ -3093,7 +3095,7 @@
         <v>0.30249999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="36">
         <v>650</v>
       </c>
@@ -3110,19 +3112,19 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>0.3</v>
       </c>
@@ -3133,17 +3135,17 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.69140625" customWidth="1"/>
+    <col min="3" max="3" width="11.15234375" customWidth="1"/>
+    <col min="4" max="4" width="10.84375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -3169,13 +3171,13 @@
         <v>31</v>
       </c>
       <c r="I1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" t="s">
         <v>32</v>
       </c>
-      <c r="J1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3207,7 +3209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>0.01</v>
       </c>
@@ -3239,7 +3241,7 @@
         <v>20.002379999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>1.9997999999999998E-2</v>
       </c>
@@ -3271,7 +3273,7 @@
         <v>40.009529999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>2.9996999999999999E-2</v>
       </c>
@@ -3303,7 +3305,7 @@
         <v>60.021769999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>4.0016999999999997E-2</v>
       </c>
@@ -3335,7 +3337,7 @@
         <v>80.043999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>5.0168999999999998E-2</v>
       </c>
@@ -3367,7 +3369,7 @@
         <v>100.11318</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>6.0899000000000002E-2</v>
       </c>
@@ -3399,7 +3401,7 @@
         <v>120.4113</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>7.3584999999999998E-2</v>
       </c>
@@ -3431,7 +3433,7 @@
         <v>141.61183</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>9.1795000000000002E-2</v>
       </c>
@@ -3463,7 +3465,7 @@
         <v>153.09189000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>0.12364700000000001</v>
       </c>
@@ -3495,7 +3497,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>0.185861</v>
       </c>
@@ -3527,7 +3529,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>0.31024499999999999</v>
       </c>
@@ -3559,7 +3561,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>0.553481</v>
       </c>
@@ -3591,7 +3593,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>1.011009</v>
       </c>
@@ -3623,7 +3625,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>1.3649899999999999</v>
       </c>
@@ -3655,7 +3657,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>1.8353809999999999</v>
       </c>
@@ -3694,11 +3696,11 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -3718,7 +3720,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3738,7 +3740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>0.01</v>
       </c>
@@ -3758,7 +3760,7 @@
         <v>20.00216</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>1.9997999999999998E-2</v>
       </c>
@@ -3778,7 +3780,7 @@
         <v>40.008650000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>2.9996999999999999E-2</v>
       </c>
@@ -3798,7 +3800,7 @@
         <v>60.019509999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>4.0016999999999997E-2</v>
       </c>
@@ -3818,7 +3820,7 @@
         <v>80.03546</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>5.0168999999999998E-2</v>
       </c>
@@ -3838,7 +3840,7 @@
         <v>100.06189999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>6.0899000000000002E-2</v>
       </c>
@@ -3858,7 +3860,7 @@
         <v>120.1255</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>7.3584999999999998E-2</v>
       </c>
@@ -3878,7 +3880,7 @@
         <v>140.32470000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>9.1795000000000002E-2</v>
       </c>
@@ -3898,7 +3900,7 @@
         <v>160.95769999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>0.12364700000000001</v>
       </c>
@@ -3918,7 +3920,7 @@
         <v>171.64840000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>0.185861</v>
       </c>
@@ -3938,7 +3940,7 @@
         <v>191.94120000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>0.31024499999999999</v>
       </c>
@@ -3958,7 +3960,7 @@
         <v>595.16099999999994</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>0.553481</v>
       </c>
@@ -3978,7 +3980,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>1.011009</v>
       </c>
@@ -3998,7 +4000,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>1.3649899999999999</v>
       </c>
@@ -4018,7 +4020,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>1.8353809999999999</v>
       </c>
@@ -4038,7 +4040,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>50.319659999999999</v>
       </c>
@@ -4065,18 +4067,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="2"/>
-    <col min="2" max="2" width="12.7109375" style="2" customWidth="1"/>
-    <col min="3" max="6" width="8.85546875" style="2"/>
-    <col min="7" max="7" width="24.140625" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="1" width="8.84375" style="2"/>
+    <col min="2" max="2" width="12.69140625" style="2" customWidth="1"/>
+    <col min="3" max="6" width="8.84375" style="2"/>
+    <col min="7" max="7" width="24.15234375" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -4084,7 +4086,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>20</v>
       </c>
@@ -4092,7 +4094,7 @@
         <v>1.5299999999999999E-5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>50</v>
       </c>
@@ -4100,7 +4102,7 @@
         <v>1.5500000000000001E-5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>100</v>
       </c>
@@ -4108,7 +4110,7 @@
         <v>1.59E-5</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>150</v>
       </c>
@@ -4122,7 +4124,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>200</v>
       </c>
@@ -4130,7 +4132,7 @@
         <v>1.66E-5</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>250</v>
       </c>
@@ -4138,7 +4140,7 @@
         <v>1.6900000000000001E-5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>300</v>
       </c>
@@ -4146,7 +4148,7 @@
         <v>1.7200000000000001E-5</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>350</v>
       </c>
@@ -4154,7 +4156,7 @@
         <v>1.7499999999999998E-5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>400</v>
       </c>
@@ -4162,7 +4164,7 @@
         <v>1.7E-5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>450</v>
       </c>
@@ -4170,7 +4172,7 @@
         <v>1.8E-5</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>500</v>
       </c>
@@ -4178,7 +4180,7 @@
         <v>1.8300000000000001E-5</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>550</v>
       </c>
@@ -4186,7 +4188,7 @@
         <v>1.8499999999999999E-5</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>600</v>
       </c>
@@ -4194,7 +4196,7 @@
         <v>1.8700000000000001E-5</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>650</v>
       </c>
@@ -4202,7 +4204,7 @@
         <v>1.8899999999999999E-5</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
         <v>700</v>
       </c>
@@ -4210,7 +4212,7 @@
         <v>1.9000000000000001E-5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
         <v>750</v>
       </c>
@@ -4218,7 +4220,7 @@
         <v>1.9199999999999999E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>800</v>
       </c>
@@ -4226,7 +4228,7 @@
         <v>1.9300000000000002E-5</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>850</v>
       </c>
@@ -4234,7 +4236,7 @@
         <v>1.95E-5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
         <v>900</v>
       </c>
@@ -4242,7 +4244,7 @@
         <v>1.9599999999999999E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A21" s="2">
         <v>950</v>
       </c>
@@ -4250,7 +4252,7 @@
         <v>1.9700000000000001E-5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A22" s="2">
         <v>1000</v>
       </c>
@@ -4265,16 +4267,16 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="6" width="8.85546875" style="2"/>
-    <col min="7" max="7" width="24.140625" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="6" width="8.84375" style="2"/>
+    <col min="7" max="7" width="24.15234375" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.84375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -4282,7 +4284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>20</v>
       </c>
@@ -4290,7 +4292,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>100</v>
       </c>
@@ -4298,7 +4300,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>150</v>
       </c>
@@ -4312,7 +4314,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>200</v>
       </c>
@@ -4320,7 +4322,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>250</v>
       </c>
@@ -4328,7 +4330,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>300</v>
       </c>
@@ -4336,7 +4338,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>350</v>
       </c>
@@ -4344,7 +4346,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>400</v>
       </c>
@@ -4352,7 +4354,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>450</v>
       </c>
@@ -4360,7 +4362,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>500</v>
       </c>
@@ -4368,7 +4370,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>550</v>
       </c>
@@ -4376,7 +4378,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>600</v>
       </c>
@@ -4384,7 +4386,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>650</v>
       </c>
@@ -4392,7 +4394,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>700</v>
       </c>
@@ -4407,14 +4409,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4422,14 +4424,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="84" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="84"/>
       <c r="C2" s="84"/>
     </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
         <v>23</v>
       </c>
@@ -4438,7 +4440,7 @@
       </c>
       <c r="C3" s="83"/>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
@@ -4449,7 +4451,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="11">
         <v>10</v>
       </c>
@@ -4460,7 +4462,7 @@
         <v>2.552</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="11">
         <v>20</v>
       </c>
@@ -4471,7 +4473,7 @@
         <v>1.931</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="11">
         <v>40</v>
       </c>
@@ -4482,7 +4484,7 @@
         <v>1.4850000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="11">
         <v>100</v>
       </c>
@@ -4493,7 +4495,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="11">
         <v>200</v>
       </c>
@@ -4504,7 +4506,7 @@
         <v>0.86899999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="11">
         <v>400</v>
       </c>
@@ -4515,7 +4517,7 @@
         <v>0.71499999999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="11">
         <v>1000</v>
       </c>
@@ -4526,7 +4528,7 @@
         <v>0.57799999999999996</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="11">
         <v>2000</v>
       </c>
@@ -4537,7 +4539,7 @@
         <v>0.48799999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="11">
         <v>4000</v>
       </c>
@@ -4548,7 +4550,7 @@
         <v>0.41199999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="11">
         <v>10000</v>
       </c>
@@ -4559,7 +4561,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="11">
         <v>20000</v>
       </c>
@@ -4570,7 +4572,7 @@
         <v>0.28199999999999997</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="11">
         <v>40000</v>
       </c>
@@ -4581,7 +4583,7 @@
         <v>0.249</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" s="11">
         <v>100000</v>
       </c>
@@ -4592,7 +4594,7 @@
         <v>0.221</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" s="11">
         <v>200000</v>
       </c>
@@ -4603,7 +4605,7 @@
         <v>0.20699999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="11">
         <v>400000</v>
       </c>
@@ -4614,7 +4616,7 @@
         <v>0.19700000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="11">
         <v>1000000</v>
       </c>
@@ -4625,7 +4627,7 @@
         <v>0.186</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="11">
         <v>5000000</v>
       </c>
@@ -4636,7 +4638,7 @@
         <v>0.16800000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="11">
         <v>10000000</v>
       </c>
@@ -4647,7 +4649,7 @@
         <v>0.159</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="11">
         <v>50000000</v>
       </c>
@@ -4658,7 +4660,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A24" s="12">
         <v>100000000</v>
       </c>
@@ -4679,28 +4681,28 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="3" max="3" width="10.85546875" customWidth="1"/>
+    <col min="3" max="3" width="10.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15.45" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="87" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="88"/>
       <c r="C1" s="89"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="51"/>
       <c r="B2" s="85" t="s">
         <v>15</v>
       </c>
       <c r="C2" s="86"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="46" t="s">
         <v>13</v>
       </c>
@@ -4711,7 +4713,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="47">
         <v>20</v>
       </c>
@@ -4723,7 +4725,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="48">
         <v>50</v>
       </c>
@@ -4735,7 +4737,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="48">
         <v>75</v>
       </c>
@@ -4747,7 +4749,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" s="48">
         <v>100</v>
       </c>
@@ -4760,7 +4762,7 @@
       </c>
       <c r="H7" s="79"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" s="48">
         <v>125</v>
       </c>
@@ -4772,7 +4774,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" s="48">
         <v>150</v>
       </c>
@@ -4784,7 +4786,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A10" s="48">
         <v>175</v>
       </c>
@@ -4796,7 +4798,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" s="48">
         <v>200</v>
       </c>
@@ -4808,7 +4810,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12" s="48">
         <v>225</v>
       </c>
@@ -4820,7 +4822,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" s="48">
         <v>250</v>
       </c>
@@ -4832,7 +4834,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="48">
         <v>275</v>
       </c>
@@ -4844,7 +4846,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15" s="48">
         <v>300</v>
       </c>
@@ -4856,7 +4858,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A16" s="48">
         <v>325</v>
       </c>
@@ -4868,7 +4870,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" s="48">
         <v>350</v>
       </c>
@@ -4880,7 +4882,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" s="48">
         <v>375</v>
       </c>
@@ -4892,7 +4894,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="48">
         <v>400</v>
       </c>
@@ -4904,7 +4906,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="48">
         <v>425</v>
       </c>
@@ -4916,7 +4918,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="48">
         <v>450</v>
       </c>
@@ -4928,7 +4930,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="48">
         <v>475</v>
       </c>
@@ -4940,7 +4942,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="48">
         <v>500</v>
       </c>
@@ -4952,7 +4954,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="48">
         <v>525</v>
       </c>
@@ -4964,7 +4966,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="48">
         <v>550</v>
       </c>
@@ -4976,7 +4978,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" s="48">
         <v>575</v>
       </c>
@@ -4988,7 +4990,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" s="48">
         <v>600</v>
       </c>
@@ -5000,7 +5002,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="49">
         <v>625</v>
       </c>
@@ -5012,7 +5014,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="49">
         <v>650</v>
       </c>
@@ -5024,7 +5026,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="49">
         <v>675</v>
       </c>
@@ -5047,21 +5049,21 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="8.84375" style="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.85546875" style="1"/>
+    <col min="3" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A1" s="53" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
       <c r="B2" s="81" t="s">
         <v>16</v>
       </c>
@@ -5076,7 +5078,7 @@
       <c r="K2" s="81"/>
       <c r="L2" s="81"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A3" s="53" t="s">
         <v>13</v>
       </c>
@@ -5114,7 +5116,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A4" s="77">
         <v>0</v>
       </c>
@@ -5152,7 +5154,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A5" s="53">
         <v>50</v>
       </c>
@@ -5190,7 +5192,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A6" s="53">
         <v>100</v>
       </c>
@@ -5228,7 +5230,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A7" s="53">
         <v>150</v>
       </c>
@@ -5266,7 +5268,7 @@
         <v>1.22</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A8" s="53">
         <v>200</v>
       </c>
@@ -5304,7 +5306,7 @@
         <v>1.21</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A9" s="53">
         <v>250</v>
       </c>
@@ -5342,7 +5344,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A10" s="53">
         <v>300</v>
       </c>
@@ -5380,7 +5382,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" s="53">
         <v>350</v>
       </c>
@@ -5428,20 +5430,20 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AW18"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="13.28515625" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="2" width="13.3046875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.4">
       <c r="C2" s="81" t="s">
         <v>16</v>
       </c>
@@ -5483,7 +5485,7 @@
       <c r="AM2" s="81"/>
       <c r="AN2" s="81"/>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A3" s="53" t="s">
         <v>13</v>
       </c>
@@ -5632,7 +5634,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>20</v>
       </c>
@@ -5781,7 +5783,7 @@
         <v>537.86510999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>80</v>
       </c>
@@ -5930,7 +5932,7 @@
         <v>537.86510999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>100</v>
       </c>
@@ -6079,7 +6081,7 @@
         <v>537.86510999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>125</v>
       </c>
@@ -6228,7 +6230,7 @@
         <v>537.86510999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>150</v>
       </c>
@@ -6377,7 +6379,7 @@
         <v>537.86510999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>175</v>
       </c>
@@ -6526,7 +6528,7 @@
         <v>537.86510999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>227</v>
       </c>
@@ -6675,7 +6677,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>283.5</v>
       </c>
@@ -6824,7 +6826,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>340</v>
       </c>
@@ -6973,7 +6975,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>350</v>
       </c>
@@ -7122,7 +7124,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>375</v>
       </c>
@@ -7271,7 +7273,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>400</v>
       </c>
@@ -7420,7 +7422,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>425</v>
       </c>
@@ -7569,7 +7571,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>450</v>
       </c>
@@ -7718,7 +7720,7 @@
         <v>703.098614072705</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>475</v>
       </c>
@@ -7877,25 +7879,25 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
       <c r="B2" s="81" t="s">
         <v>16</v>
       </c>
       <c r="C2" s="81"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="53" t="s">
         <v>13</v>
       </c>
@@ -7906,7 +7908,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>20</v>
       </c>
@@ -7917,7 +7919,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>100</v>
       </c>
@@ -7928,7 +7930,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>150</v>
       </c>
@@ -7939,7 +7941,7 @@
         <v>177.5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>200</v>
       </c>
@@ -7950,7 +7952,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>250</v>
       </c>
@@ -7961,7 +7963,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>300</v>
       </c>
@@ -7972,7 +7974,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>350</v>
       </c>
@@ -7983,7 +7985,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>400</v>
       </c>
@@ -7994,7 +7996,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>450</v>
       </c>
@@ -8005,7 +8007,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>500</v>
       </c>
@@ -8016,7 +8018,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>550</v>
       </c>
@@ -8027,7 +8029,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>1000</v>
       </c>
@@ -8047,14 +8049,14 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:AW18"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="16384" width="8.84375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A1" s="81" t="s">
         <v>17</v>
       </c>
@@ -8073,7 +8075,7 @@
       <c r="N1" s="81"/>
       <c r="O1" s="81"/>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.4">
       <c r="B2" s="81" t="s">
         <v>16</v>
       </c>
@@ -8125,7 +8127,7 @@
       <c r="AV2" s="81"/>
       <c r="AW2" s="81"/>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -8274,7 +8276,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>20</v>
       </c>
@@ -8423,7 +8425,7 @@
         <v>615.75505199157828</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>80</v>
       </c>
@@ -8572,7 +8574,7 @@
         <v>615.75505199157828</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>100</v>
       </c>
@@ -8721,7 +8723,7 @@
         <v>615.75505199157828</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>125</v>
       </c>
@@ -8870,7 +8872,7 @@
         <v>615.75505199157828</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>150</v>
       </c>
@@ -9019,7 +9021,7 @@
         <v>615.75505199157828</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>175</v>
       </c>
@@ -9168,7 +9170,7 @@
         <v>615.75505199157828</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>227</v>
       </c>
@@ -9317,7 +9319,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>283.5</v>
       </c>
@@ -9466,7 +9468,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>340</v>
       </c>
@@ -9615,7 +9617,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>350</v>
       </c>
@@ -9764,7 +9766,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>375</v>
       </c>
@@ -9913,7 +9915,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>400</v>
       </c>
@@ -10062,7 +10064,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>425</v>
       </c>
@@ -10211,7 +10213,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>450</v>
       </c>
@@ -10360,7 +10362,7 @@
         <v>718.59707075261247</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>475</v>
       </c>
@@ -10520,26 +10522,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="f41f4605-e15c-4135-bd96-d3970596b173" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71e126cb-1963-4e7b-b13a-15d2f64f78e9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100EFE0C39B20CFE747B2EDBEF1A424A9C1" ma:contentTypeVersion="14" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="fc5d43efe255f0326fdf88779d9e8cc0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71e126cb-1963-4e7b-b13a-15d2f64f78e9" xmlns:ns3="f41f4605-e15c-4135-bd96-d3970596b173" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c67b044c92a952204dd5da40bf3ff3c1" ns2:_="" ns3:_="">
     <xsd:import namespace="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
@@ -10768,10 +10750,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="f41f4605-e15c-4135-bd96-d3970596b173" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71e126cb-1963-4e7b-b13a-15d2f64f78e9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1EB181C-B032-4B55-8488-B934A42A5264}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50B0D253-82BE-407B-A99A-5C9012782B82}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
+    <ds:schemaRef ds:uri="f41f4605-e15c-4135-bd96-d3970596b173"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10781,10 +10794,16 @@
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f41f4605-e15c-4135-bd96-d3970596b173"/>
+    <ds:schemaRef ds:uri="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50B0D253-82BE-407B-A99A-5C9012782B82}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1EB181C-B032-4B55-8488-B934A42A5264}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>